<commit_message>
feat(office): stabilize preview packages
Unify packages under @arcships and add instance-owned runtimes, resource limits, public assets, and reproducible release checks.

Bring DOCX, XLSX, and PDF demo behavior in line with production preview paths, including worker fidelity and browser acceptance tests.
</commit_message>
<xml_diff>
--- a/apps/demo/public/samples/charts-images.xlsx
+++ b/apps/demo/public/samples/charts-images.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revenue Chart" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,6 +29,10 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001C3A5E"/>
     </font>
   </fonts>
   <fills count="3">
@@ -55,10 +60,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -233,6 +241,109 @@
 </chartSpace>
 </file>
 
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Revenue by Quarter</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Dashboard'!B1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Dashboard'!$A$2:$A$5</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Dashboard'!$B$2:$B$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Revenue</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/chartsheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartsheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</chartsheet>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
@@ -282,6 +393,28 @@
     </pic>
     <clientData/>
   </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <absoluteAnchor>
+    <pos x="0" y="0"/>
+    <ext cx="0" cy="0"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </absoluteAnchor>
 </wsDr>
 </file>
 
@@ -574,7 +707,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -646,7 +779,18 @@
         <v>410</v>
       </c>
     </row>
+    <row r="7" ht="28" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Worker merged region — image and merge parity</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="28" customHeight="1"/>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A7:C8"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(office): complete preview fidelity
Render DOCX notes and searchable document results.

Show XLSX links, comments, conditional visuals, sparklines, shapes, and controls in the viewer and Demo.
</commit_message>
<xml_diff>
--- a/apps/demo/public/samples/charts-images.xlsx
+++ b/apps/demo/public/samples/charts-images.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -33,6 +33,13 @@
     <font>
       <b val="1"/>
       <color rgb="001C3A5E"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="10"/>
+      <sz val="12"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -57,20 +64,24 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -344,6 +355,25 @@
 </chartsheet>
 </file>
 
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>财务审核</author>
+  </authors>
+  <commentList>
+    <comment ref="B2" authorId="0" shapeId="0">
+      <text>
+        <t>该季度收入已通过财务复核。</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/ctrlProps/ctrlProp1.xml><?xml version="1.0" encoding="utf-8"?>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="1" fmlaLink="Dashboard!$A$10"/>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
@@ -393,6 +423,51 @@
     </pic>
     <clientData/>
   </oneCellAnchor>
+  <xdr:twoCellAnchor xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp>
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="9002" name="审批提醒" descr="只读形状展示"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:solidFill>
+          <a:srgbClr val="DBEAFE"/>
+        </a:solidFill>
+        <a:ln w="19050">
+          <a:solidFill>
+            <a:srgbClr val="2563EB"/>
+          </a:solidFill>
+        </a:ln>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="zh-CN" sz="1200" b="1"/>
+            <a:t>审批提醒：请核对季度收入</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </wsDr>
 </file>
 
@@ -707,7 +782,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -726,9 +801,14 @@
           <t>Exceptions</t>
         </is>
       </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>趋势</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>Q1</t>
         </is>
@@ -752,6 +832,9 @@
       <c r="C3" t="n">
         <v>690</v>
       </c>
+      <c r="D3" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -765,6 +848,9 @@
       <c r="C4" t="n">
         <v>540</v>
       </c>
+      <c r="D4" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -778,9 +864,12 @@
       <c r="C5" t="n">
         <v>410</v>
       </c>
+      <c r="D5" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="7" ht="28" customHeight="1">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Worker merged region — image and merge parity</t>
         </is>
@@ -791,7 +880,77 @@
   <mergeCells count="1">
     <mergeCell ref="A7:C8"/>
   </mergeCells>
+  <conditionalFormatting sqref="B2:B5">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C2:C5">
+    <cfRule type="dataBar" priority="2">
+      <dataBar showValue="1">
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="005B9BD5"/>
+      </dataBar>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D3:D5">
+    <cfRule type="iconSet" priority="3">
+      <iconSet iconSet="3TrafficLights1" showValue="1">
+        <cfvo type="num" val="1"/>
+        <cfvo type="num" val="2"/>
+        <cfvo type="num" val="3"/>
+      </iconSet>
+    </cfRule>
+  </conditionalFormatting>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+  <extLst>
+    <ext uri="{05C60535-1F16-4fd2-B633-F4F36F0B64E0}">
+      <x14:sparklineGroups xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+        <x14:sparklineGroup type="line" markers="1">
+          <x14:colorSeries rgb="FF2563EB"/>
+          <x14:colorMarkers rgb="FFDC2626"/>
+          <x14:sparklines>
+            <x14:sparkline>
+              <xm:f>Dashboard!B2:B5</xm:f>
+              <xm:sqref>D2</xm:sqref>
+            </x14:sparkline>
+          </x14:sparklines>
+        </x14:sparklineGroup>
+      </x14:sparklineGroups>
+    </ext>
+  </extLst>
+  <controls>
+    <control xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" shapeId="9001" name="发布前确认" r:id="rIdFidelityControl">
+      <controlPr>
+        <xdr:anchor xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+          <xdr:from>
+            <xdr:col>0</xdr:col>
+            <xdr:colOff>0</xdr:colOff>
+            <xdr:row>9</xdr:row>
+            <xdr:rowOff>0</xdr:rowOff>
+          </xdr:from>
+          <xdr:to>
+            <xdr:col>2</xdr:col>
+            <xdr:colOff>0</xdr:colOff>
+            <xdr:row>11</xdr:row>
+            <xdr:rowOff>0</xdr:rowOff>
+          </xdr:to>
+        </xdr:anchor>
+      </controlPr>
+    </control>
+  </controls>
 </worksheet>
 </file>
</xml_diff>